<commit_message>
Rebalance: Substrate 42 / Compute 34 / Materials 2 / Ballast 22
Energy renamed to Substrate (fuel, molecules, ground, grid equipment) and
adds ETN 2 and HUBB 2. Compute adds ASML 2. RARA11.SA cut to 2. Ballast:
AVDV 4, JPM 4, IEUR 4 added (MSCI Europe IMI; 4.34% ASML vs EXSA 4.41%),
XLP removed. NBIS/CRWV classification-stretch disclosures removed.
Falsification notes for ETN, HUBB, ASML, IEUR, RARA11 and the XLP removal.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/research/verification.xlsx
+++ b/research/verification.xlsx
@@ -735,7 +735,7 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Snapshot as of 2026-10-14 19:21 UTC</t>
+          <t>Snapshot as of 2026-10-14 19:56 UTC</t>
         </is>
       </c>
     </row>
@@ -6081,7 +6081,7 @@
         </is>
       </c>
       <c r="H9" t="n">
-        <v>30.45733205672228</v>
+        <v>30.45734581100089</v>
       </c>
     </row>
     <row r="10">
@@ -6127,7 +6127,7 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Snapshot as of 2026-10-14 19:21 UTC</t>
+          <t>Snapshot as of 2026-10-14 19:56 UTC</t>
         </is>
       </c>
     </row>
@@ -6138,7 +6138,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>27.33520126342773</v>
+        <v>27.3351993560791</v>
       </c>
       <c r="C12" t="n">
         <v>5.373300075531006</v>
@@ -6180,7 +6180,7 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>27.24405097961426</v>
+        <v>27.24405288696289</v>
       </c>
       <c r="C14" t="n">
         <v>5.357800006866455</v>
@@ -6222,7 +6222,7 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>27.43546485900879</v>
+        <v>27.43546295166016</v>
       </c>
       <c r="C16" t="n">
         <v>5.374599933624268</v>
@@ -6264,7 +6264,7 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>28.11907196044922</v>
+        <v>28.11907386779785</v>
       </c>
       <c r="C18" t="n">
         <v>5.395899772644043</v>
@@ -6327,7 +6327,7 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>29.49540519714355</v>
+        <v>29.49540328979492</v>
       </c>
       <c r="C21" t="n">
         <v>5.330900192260742</v>
@@ -6348,7 +6348,7 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>30.26104354858398</v>
+        <v>30.26104545593262</v>
       </c>
       <c r="C22" t="n">
         <v>5.289700031280518</v>
@@ -6411,7 +6411,7 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>29.8053035736084</v>
+        <v>29.80530548095703</v>
       </c>
       <c r="C25" t="n">
         <v>5.296500205993652</v>
@@ -6432,7 +6432,7 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>29.96937370300293</v>
+        <v>29.9693717956543</v>
       </c>
       <c r="C26" t="n">
         <v>5.295599937438965</v>
@@ -6495,7 +6495,7 @@
         </is>
       </c>
       <c r="B29" t="n">
-        <v>29.68680953979492</v>
+        <v>29.68681335449219</v>
       </c>
       <c r="C29" t="n">
         <v>5.332300186157227</v>
@@ -6537,7 +6537,7 @@
         </is>
       </c>
       <c r="B31" t="n">
-        <v>29.42248344421387</v>
+        <v>29.42248153686523</v>
       </c>
       <c r="C31" t="n">
         <v>5.386799812316895</v>
@@ -6579,7 +6579,7 @@
         </is>
       </c>
       <c r="B33" t="n">
-        <v>29.53186416625977</v>
+        <v>29.53186225891113</v>
       </c>
       <c r="C33" t="n">
         <v>5.33080005645752</v>
@@ -6621,7 +6621,7 @@
         </is>
       </c>
       <c r="B35" t="n">
-        <v>29.03055000305176</v>
+        <v>29.03055191040039</v>
       </c>
       <c r="C35" t="n">
         <v>5.335400104522705</v>
@@ -6684,7 +6684,7 @@
         </is>
       </c>
       <c r="B38" t="n">
-        <v>29.6412410736084</v>
+        <v>29.64123916625977</v>
       </c>
       <c r="C38" t="n">
         <v>5.306099891662598</v>
@@ -6768,7 +6768,7 @@
         </is>
       </c>
       <c r="B42" t="n">
-        <v>29.11258316040039</v>
+        <v>29.11258125305176</v>
       </c>
       <c r="C42" t="n">
         <v>5.43149995803833</v>
@@ -6789,7 +6789,7 @@
         </is>
       </c>
       <c r="B43" t="n">
-        <v>28.6294994354248</v>
+        <v>28.62950134277344</v>
       </c>
       <c r="C43" t="n">
         <v>5.469799995422363</v>
@@ -6852,7 +6852,7 @@
         </is>
       </c>
       <c r="B46" t="n">
-        <v>28.01880836486816</v>
+        <v>28.0188102722168</v>
       </c>
       <c r="C46" t="n">
         <v>5.413400173187256</v>
@@ -6873,7 +6873,7 @@
         </is>
       </c>
       <c r="B47" t="n">
-        <v>28.32871437072754</v>
+        <v>28.32871246337891</v>
       </c>
       <c r="C47" t="n">
         <v>5.507500171661377</v>
@@ -6894,7 +6894,7 @@
         </is>
       </c>
       <c r="B48" t="n">
-        <v>28.16464614868164</v>
+        <v>28.16464424133301</v>
       </c>
       <c r="C48" t="n">
         <v>5.518499851226807</v>
@@ -6936,7 +6936,7 @@
         </is>
       </c>
       <c r="B50" t="n">
-        <v>28.34694290161133</v>
+        <v>28.3469409942627</v>
       </c>
       <c r="C50" t="n">
         <v>5.53980016708374</v>
@@ -6957,7 +6957,7 @@
         </is>
       </c>
       <c r="B51" t="n">
-        <v>28.49938201904297</v>
+        <v>28.4993839263916</v>
       </c>
       <c r="C51" t="n">
         <v>5.590000152587891</v>
@@ -6999,7 +6999,7 @@
         </is>
       </c>
       <c r="B53" t="n">
-        <v>28.8942928314209</v>
+        <v>28.89429473876953</v>
       </c>
       <c r="C53" t="n">
         <v>5.542500019073486</v>
@@ -7083,7 +7083,7 @@
         </is>
       </c>
       <c r="B57" t="n">
-        <v>27.86940765380859</v>
+        <v>27.86940574645996</v>
       </c>
       <c r="C57" t="n">
         <v>5.40749979019165</v>
@@ -7146,7 +7146,7 @@
         </is>
       </c>
       <c r="B60" t="n">
-        <v>28.48998069763184</v>
+        <v>28.48998260498047</v>
       </c>
       <c r="C60" t="n">
         <v>5.386600017547607</v>
@@ -7167,7 +7167,7 @@
         </is>
       </c>
       <c r="B61" t="n">
-        <v>28.54640007019043</v>
+        <v>28.54639625549316</v>
       </c>
       <c r="C61" t="n">
         <v>5.370299816131592</v>
@@ -7209,7 +7209,7 @@
         </is>
       </c>
       <c r="B63" t="n">
-        <v>30.07902526855469</v>
+        <v>30.07902717590332</v>
       </c>
       <c r="C63" t="n">
         <v>5.371300220489502</v>
@@ -7251,7 +7251,7 @@
         </is>
       </c>
       <c r="B65" t="n">
-        <v>30.12604141235352</v>
+        <v>30.12603950500488</v>
       </c>
       <c r="C65" t="n">
         <v>5.367899894714355</v>
@@ -7272,7 +7272,7 @@
         </is>
       </c>
       <c r="B66" t="n">
-        <v>30.2482738494873</v>
+        <v>30.24827003479004</v>
       </c>
       <c r="C66" t="n">
         <v>5.367700099945068</v>
@@ -7293,7 +7293,7 @@
         </is>
       </c>
       <c r="B67" t="n">
-        <v>30.36110496520996</v>
+        <v>30.36110687255859</v>
       </c>
       <c r="C67" t="n">
         <v>5.36870002746582</v>
@@ -7314,7 +7314,7 @@
         </is>
       </c>
       <c r="B68" t="n">
-        <v>31.43300819396973</v>
+        <v>31.43300437927246</v>
       </c>
       <c r="C68" t="n">
         <v>5.374300003051758</v>
@@ -7335,7 +7335,7 @@
         </is>
       </c>
       <c r="B69" t="n">
-        <v>31.57404899597168</v>
+        <v>31.57404708862305</v>
       </c>
       <c r="C69" t="n">
         <v>5.31879997253418</v>
@@ -7482,7 +7482,7 @@
         </is>
       </c>
       <c r="B76" t="n">
-        <v>35.01541137695312</v>
+        <v>35.01540756225586</v>
       </c>
       <c r="C76" t="n">
         <v>5.255000114440918</v>
@@ -7524,7 +7524,7 @@
         </is>
       </c>
       <c r="B78" t="n">
-        <v>35.27868270874023</v>
+        <v>35.2786865234375</v>
       </c>
       <c r="C78" t="n">
         <v>5.237500190734863</v>
@@ -7545,7 +7545,7 @@
         </is>
       </c>
       <c r="B79" t="n">
-        <v>34.78974914550781</v>
+        <v>34.78974533081055</v>
       </c>
       <c r="C79" t="n">
         <v>5.23799991607666</v>
@@ -7587,7 +7587,7 @@
         </is>
       </c>
       <c r="B81" t="n">
-        <v>35.09063339233398</v>
+        <v>35.09062957763672</v>
       </c>
       <c r="C81" t="n">
         <v>5.21589994430542</v>
@@ -7608,7 +7608,7 @@
         </is>
       </c>
       <c r="B82" t="n">
-        <v>35.11883926391602</v>
+        <v>35.11883544921875</v>
       </c>
       <c r="C82" t="n">
         <v>5.19159984588623</v>
@@ -7629,7 +7629,7 @@
         </is>
       </c>
       <c r="B83" t="n">
-        <v>35.80523300170898</v>
+        <v>35.80522918701172</v>
       </c>
       <c r="C83" t="n">
         <v>5.196199893951416</v>
@@ -7650,7 +7650,7 @@
         </is>
       </c>
       <c r="B84" t="n">
-        <v>34.8931770324707</v>
+        <v>34.89317321777344</v>
       </c>
       <c r="C84" t="n">
         <v>5.198699951171875</v>
@@ -7671,7 +7671,7 @@
         </is>
       </c>
       <c r="B85" t="n">
-        <v>34.68631744384766</v>
+        <v>34.68631362915039</v>
       </c>
       <c r="C85" t="n">
         <v>5.213900089263916</v>
@@ -7713,7 +7713,7 @@
         </is>
       </c>
       <c r="B87" t="n">
-        <v>35.55136108398438</v>
+        <v>35.55135726928711</v>
       </c>
       <c r="C87" t="n">
         <v>5.234399795532227</v>
@@ -7839,7 +7839,7 @@
         </is>
       </c>
       <c r="B93" t="n">
-        <v>36.98056411743164</v>
+        <v>36.98056030273438</v>
       </c>
       <c r="C93" t="n">
         <v>5.136600017547607</v>
@@ -7881,7 +7881,7 @@
         </is>
       </c>
       <c r="B95" t="n">
-        <v>38.50378799438477</v>
+        <v>38.5037841796875</v>
       </c>
       <c r="C95" t="n">
         <v>5.170300006866455</v>
@@ -7965,7 +7965,7 @@
         </is>
       </c>
       <c r="B99" t="n">
-        <v>40.58177185058594</v>
+        <v>40.58176803588867</v>
       </c>
       <c r="C99" t="n">
         <v>5.243500232696533</v>
@@ -8007,7 +8007,7 @@
         </is>
       </c>
       <c r="B101" t="n">
-        <v>42.12379837036133</v>
+        <v>42.12380218505859</v>
       </c>
       <c r="C101" t="n">
         <v>5.162399768829346</v>
@@ -8028,7 +8028,7 @@
         </is>
       </c>
       <c r="B102" t="n">
-        <v>42.31185531616211</v>
+        <v>42.31185150146484</v>
       </c>
       <c r="C102" t="n">
         <v>5.151400089263916</v>
@@ -8049,7 +8049,7 @@
         </is>
       </c>
       <c r="B103" t="n">
-        <v>42.00156402587891</v>
+        <v>42.00156784057617</v>
       </c>
       <c r="C103" t="n">
         <v>5.243899822235107</v>
@@ -8070,7 +8070,7 @@
         </is>
       </c>
       <c r="B104" t="n">
-        <v>43.1204833984375</v>
+        <v>43.12047958374023</v>
       </c>
       <c r="C104" t="n">
         <v>5.329100131988525</v>
@@ -8091,7 +8091,7 @@
         </is>
       </c>
       <c r="B105" t="n">
-        <v>43.60941696166992</v>
+        <v>43.60942077636719</v>
       </c>
       <c r="C105" t="n">
         <v>5.233399868011475</v>
@@ -8154,7 +8154,7 @@
         </is>
       </c>
       <c r="B108" t="n">
-        <v>42.94182586669922</v>
+        <v>42.94182968139648</v>
       </c>
       <c r="C108" t="n">
         <v>5.219900131225586</v>
@@ -8175,7 +8175,7 @@
         </is>
       </c>
       <c r="B109" t="n">
-        <v>43.28032302856445</v>
+        <v>43.28032684326172</v>
       </c>
       <c r="C109" t="n">
         <v>5.31190013885498</v>
@@ -8196,7 +8196,7 @@
         </is>
       </c>
       <c r="B110" t="n">
-        <v>44.44625473022461</v>
+        <v>44.44625091552734</v>
       </c>
       <c r="C110" t="n">
         <v>5.232900142669678</v>
@@ -8259,7 +8259,7 @@
         </is>
       </c>
       <c r="B113" t="n">
-        <v>46.45841217041016</v>
+        <v>46.45841598510742</v>
       </c>
       <c r="C113" t="n">
         <v>5.235099792480469</v>
@@ -8364,7 +8364,7 @@
         </is>
       </c>
       <c r="B118" t="n">
-        <v>46.01648712158203</v>
+        <v>46.0164909362793</v>
       </c>
       <c r="C118" t="n">
         <v>5.157899856567383</v>
@@ -8406,7 +8406,7 @@
         </is>
       </c>
       <c r="B120" t="n">
-        <v>43.82567977905273</v>
+        <v>43.82567596435547</v>
       </c>
       <c r="C120" t="n">
         <v>5.150599956512451</v>
@@ -8448,7 +8448,7 @@
         </is>
       </c>
       <c r="B122" t="n">
-        <v>46.10111236572266</v>
+        <v>46.10111618041992</v>
       </c>
       <c r="C122" t="n">
         <v>5.095799922943115</v>
@@ -8469,7 +8469,7 @@
         </is>
       </c>
       <c r="B123" t="n">
-        <v>46.80631256103516</v>
+        <v>46.80630874633789</v>
       </c>
       <c r="C123" t="n">
         <v>5.005000114440918</v>
@@ -8490,7 +8490,7 @@
         </is>
       </c>
       <c r="B124" t="n">
-        <v>45.01981353759766</v>
+        <v>45.01980972290039</v>
       </c>
       <c r="C124" t="n">
         <v>4.994400024414062</v>
@@ -8532,7 +8532,7 @@
         </is>
       </c>
       <c r="B126" t="n">
-        <v>45.67799758911133</v>
+        <v>45.67800140380859</v>
       </c>
       <c r="C126" t="n">
         <v>4.992400169372559</v>
@@ -8595,7 +8595,7 @@
         </is>
       </c>
       <c r="B129" t="n">
-        <v>44.82235336303711</v>
+        <v>44.82235717773438</v>
       </c>
       <c r="C129" t="n">
         <v>5.007999897003174</v>
@@ -8700,7 +8700,7 @@
         </is>
       </c>
       <c r="B134" t="n">
-        <v>46.6846923828125</v>
+        <v>46.68469619750977</v>
       </c>
       <c r="C134" t="n">
         <v>4.99429988861084</v>
@@ -8721,7 +8721,7 @@
         </is>
       </c>
       <c r="B135" t="n">
-        <v>46.79912185668945</v>
+        <v>46.79911804199219</v>
       </c>
       <c r="C135" t="n">
         <v>5.017499923706055</v>
@@ -8742,7 +8742,7 @@
         </is>
       </c>
       <c r="B136" t="n">
-        <v>47.04703521728516</v>
+        <v>47.04703903198242</v>
       </c>
       <c r="C136" t="n">
         <v>4.951929092407227</v>
@@ -8763,7 +8763,7 @@
         </is>
       </c>
       <c r="B137" t="n">
-        <v>46.39863586425781</v>
+        <v>46.39863967895508</v>
       </c>
       <c r="C137" t="n">
         <v>4.984799861907959</v>
@@ -8868,7 +8868,7 @@
         </is>
       </c>
       <c r="B142" t="n">
-        <v>43.55712890625</v>
+        <v>43.55712509155273</v>
       </c>
       <c r="C142" t="n">
         <v>4.906400203704834</v>
@@ -8931,7 +8931,7 @@
         </is>
       </c>
       <c r="B145" t="n">
-        <v>43.35688781738281</v>
+        <v>43.35688400268555</v>
       </c>
       <c r="C145" t="n">
         <v>5.00409984588623</v>
@@ -8994,7 +8994,7 @@
         </is>
       </c>
       <c r="B148" t="n">
-        <v>42.52731323242188</v>
+        <v>42.52731704711914</v>
       </c>
       <c r="C148" t="n">
         <v>5.058199882507324</v>
@@ -9015,7 +9015,7 @@
         </is>
       </c>
       <c r="B149" t="n">
-        <v>42.86104965209961</v>
+        <v>42.86105346679688</v>
       </c>
       <c r="C149" t="n">
         <v>5.01170015335083</v>
@@ -9036,7 +9036,7 @@
         </is>
       </c>
       <c r="B150" t="n">
-        <v>42.41289520263672</v>
+        <v>42.41289138793945</v>
       </c>
       <c r="C150" t="n">
         <v>5.017099857330322</v>
@@ -11456,7 +11456,7 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Snapshot as of 2026-10-14 19:21 UTC</t>
+          <t>Snapshot as of 2026-10-14 19:56 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>